<commit_message>
state: session end 2026-08-18T07:05Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -24480,7 +24480,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AP62"/>
+  <dimension ref="A1:AP63"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -31638,9 +31638,107 @@
         <v>NO TRADE</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>2026-08-18 12:32:05</v>
+      </c>
+      <c r="B63">
+        <v>1057.3</v>
+      </c>
+      <c r="C63">
+        <v>1060</v>
+      </c>
+      <c r="D63">
+        <v>0.53</v>
+      </c>
+      <c r="E63">
+        <v>1100</v>
+      </c>
+      <c r="F63">
+        <v>1050</v>
+      </c>
+      <c r="G63">
+        <v>1000</v>
+      </c>
+      <c r="H63">
+        <v>1100</v>
+      </c>
+      <c r="I63">
+        <v>1080</v>
+      </c>
+      <c r="J63">
+        <v>1120</v>
+      </c>
+      <c r="K63">
+        <v>14</v>
+      </c>
+      <c r="L63">
+        <v>2</v>
+      </c>
+      <c r="M63">
+        <v>2199750</v>
+      </c>
+      <c r="N63">
+        <v>621750</v>
+      </c>
+      <c r="O63" t="str">
+        <v>Put Unwinding 8x/358500 | Call Buying 4x/1359750 | Put Writing 1x/167250 | Call Writing 1x/556500 | Call Unwinding 1x/65250 | Call Covering 1x/314250</v>
+      </c>
+      <c r="P63">
+        <v>25.13</v>
+      </c>
+      <c r="Q63" t="str">
+        <v>Bullish</v>
+      </c>
+      <c r="R63">
+        <v>0.491</v>
+      </c>
+      <c r="S63">
+        <v>0.499</v>
+      </c>
+      <c r="T63">
+        <v>0.524</v>
+      </c>
+      <c r="U63">
+        <v>0.0052</v>
+      </c>
+      <c r="V63">
+        <v>0.279</v>
+      </c>
+      <c r="W63" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X63">
+        <v>67</v>
+      </c>
+      <c r="Y63" t="str">
+        <v>Bull Call Spread</v>
+      </c>
+      <c r="Z63">
+        <v>75</v>
+      </c>
+      <c r="AA63" t="str">
+        <v>Buy Call</v>
+      </c>
+      <c r="AB63">
+        <v>60</v>
+      </c>
+      <c r="AC63" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AD63">
+        <v>50</v>
+      </c>
+      <c r="AE63">
+        <v>50000</v>
+      </c>
+      <c r="AF63" t="str">
+        <v>NO TRADE</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AP62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AP63"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
state: session end 2026-08-19T07:05Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -38020,7 +38020,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AP45"/>
+  <dimension ref="A1:AP46"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -43272,9 +43272,107 @@
         <v>same legs already traded today</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>2026-08-19 12:32:09</v>
+      </c>
+      <c r="B46">
+        <v>1048.6</v>
+      </c>
+      <c r="C46">
+        <v>1050</v>
+      </c>
+      <c r="D46">
+        <v>0.55</v>
+      </c>
+      <c r="E46">
+        <v>1100</v>
+      </c>
+      <c r="F46">
+        <v>1050</v>
+      </c>
+      <c r="G46">
+        <v>1000</v>
+      </c>
+      <c r="H46">
+        <v>1100</v>
+      </c>
+      <c r="I46">
+        <v>1080</v>
+      </c>
+      <c r="J46">
+        <v>1120</v>
+      </c>
+      <c r="K46">
+        <v>10</v>
+      </c>
+      <c r="L46">
+        <v>5</v>
+      </c>
+      <c r="M46">
+        <v>1530000</v>
+      </c>
+      <c r="N46">
+        <v>1400250</v>
+      </c>
+      <c r="O46" t="str">
+        <v>Call Unwinding 4x/1120500 | Put Unwinding 6x/725250 | Call Covering 1x/47250 | Put Writing 1x/123750 | Call Buying 2x/633750 | Put Buying 1x/279750</v>
+      </c>
+      <c r="P46">
+        <v>23.76</v>
+      </c>
+      <c r="Q46" t="str">
+        <v>Range</v>
+      </c>
+      <c r="R46">
+        <v>0.511</v>
+      </c>
+      <c r="S46">
+        <v>0.485</v>
+      </c>
+      <c r="T46">
+        <v>0.444</v>
+      </c>
+      <c r="U46">
+        <v>0.0054</v>
+      </c>
+      <c r="V46">
+        <v>0.225</v>
+      </c>
+      <c r="W46" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X46">
+        <v>67</v>
+      </c>
+      <c r="Y46" t="str">
+        <v>Iron Condor</v>
+      </c>
+      <c r="Z46">
+        <v>70</v>
+      </c>
+      <c r="AA46" t="str">
+        <v>Bull Call Spread</v>
+      </c>
+      <c r="AB46">
+        <v>50</v>
+      </c>
+      <c r="AC46" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AD46">
+        <v>50</v>
+      </c>
+      <c r="AE46">
+        <v>50000</v>
+      </c>
+      <c r="AF46" t="str">
+        <v>NO TRADE</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AP45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AP46"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
state: session end 2026-08-20T07:05Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -49714,7 +49714,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AP62"/>
+  <dimension ref="A1:AP63"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -56902,9 +56902,137 @@
         <v>NO TRADE</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>2026-08-20 12:32:43</v>
+      </c>
+      <c r="B63">
+        <v>1047</v>
+      </c>
+      <c r="C63">
+        <v>1050</v>
+      </c>
+      <c r="D63">
+        <v>0.53</v>
+      </c>
+      <c r="E63">
+        <v>1100</v>
+      </c>
+      <c r="F63">
+        <v>1050</v>
+      </c>
+      <c r="G63">
+        <v>1000</v>
+      </c>
+      <c r="H63">
+        <v>1100</v>
+      </c>
+      <c r="I63">
+        <v>1080</v>
+      </c>
+      <c r="J63">
+        <v>1120</v>
+      </c>
+      <c r="K63">
+        <v>2</v>
+      </c>
+      <c r="L63">
+        <v>11</v>
+      </c>
+      <c r="M63">
+        <v>81000</v>
+      </c>
+      <c r="N63">
+        <v>1932000</v>
+      </c>
+      <c r="O63" t="str">
+        <v>Put Buying 2x/297750 | Call Unwinding 4x/752250 | Call Writing 2x/698250 | Put Covering 3x/183750 | Call Covering 2x/81000</v>
+      </c>
+      <c r="P63">
+        <v>23.74</v>
+      </c>
+      <c r="Q63" t="str">
+        <v>Bearish</v>
+      </c>
+      <c r="R63">
+        <v>0.502</v>
+      </c>
+      <c r="S63">
+        <v>0.494</v>
+      </c>
+      <c r="T63">
+        <v>0.408</v>
+      </c>
+      <c r="U63">
+        <v>0.0055</v>
+      </c>
+      <c r="V63">
+        <v>0.181</v>
+      </c>
+      <c r="W63" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X63">
+        <v>83</v>
+      </c>
+      <c r="Y63" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="Z63">
+        <v>100</v>
+      </c>
+      <c r="AA63" t="str">
+        <v>Buy Put</v>
+      </c>
+      <c r="AB63">
+        <v>60</v>
+      </c>
+      <c r="AC63" t="str">
+        <v>Iron Condor</v>
+      </c>
+      <c r="AD63">
+        <v>40</v>
+      </c>
+      <c r="AE63">
+        <v>50000</v>
+      </c>
+      <c r="AF63" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AG63" t="str">
+        <v>BUY 1050PE | SELL 1040PE</v>
+      </c>
+      <c r="AH63">
+        <v>1</v>
+      </c>
+      <c r="AI63">
+        <v>4.45</v>
+      </c>
+      <c r="AJ63">
+        <v>2.23</v>
+      </c>
+      <c r="AK63" t="str">
+        <v>SIGNAL</v>
+      </c>
+      <c r="AL63">
+        <v>1669</v>
+      </c>
+      <c r="AM63" t="str">
+        <v/>
+      </c>
+      <c r="AN63" t="str">
+        <v/>
+      </c>
+      <c r="AO63" t="str">
+        <v>ride</v>
+      </c>
+      <c r="AP63" t="str">
+        <v>bias Bearish persisted 1/2 polls</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AP62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AP63"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
state: session end 2026-08-24T07:05Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -12260,7 +12260,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AS59"/>
+  <dimension ref="A1:AS61"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -19595,9 +19595,283 @@
         <v>bias Range persisted 1/3 polls</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>2026-08-24 12:30:47</v>
+      </c>
+      <c r="B60">
+        <v>1034.6</v>
+      </c>
+      <c r="C60">
+        <v>1030</v>
+      </c>
+      <c r="D60">
+        <v>0.6</v>
+      </c>
+      <c r="E60">
+        <v>1000</v>
+      </c>
+      <c r="F60">
+        <v>1100</v>
+      </c>
+      <c r="G60">
+        <v>1080</v>
+      </c>
+      <c r="H60">
+        <v>1100</v>
+      </c>
+      <c r="I60">
+        <v>1080</v>
+      </c>
+      <c r="J60">
+        <v>1050</v>
+      </c>
+      <c r="K60">
+        <v>6</v>
+      </c>
+      <c r="L60">
+        <v>8</v>
+      </c>
+      <c r="M60">
+        <v>1488000</v>
+      </c>
+      <c r="N60">
+        <v>2711250</v>
+      </c>
+      <c r="O60" t="str">
+        <v>Call Unwinding 4x/1976250 | Call Covering 3x/538500 | Call Buying 1x/463500 | Put Covering 4x/735000 | Put Unwinding 2x/486000</v>
+      </c>
+      <c r="P60">
+        <v>51.56</v>
+      </c>
+      <c r="Q60" t="str">
+        <v>Bearish</v>
+      </c>
+      <c r="R60">
+        <v>0.5</v>
+      </c>
+      <c r="S60">
+        <v>0.454</v>
+      </c>
+      <c r="T60">
+        <v>2.224</v>
+      </c>
+      <c r="U60">
+        <v>0.0059</v>
+      </c>
+      <c r="V60">
+        <v>0.072</v>
+      </c>
+      <c r="W60" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X60">
+        <v>1038.8</v>
+      </c>
+      <c r="Y60">
+        <v>0.69</v>
+      </c>
+      <c r="Z60" t="str">
+        <v>Short Buildup</v>
+      </c>
+      <c r="AA60">
+        <v>83</v>
+      </c>
+      <c r="AB60" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AC60">
+        <v>100</v>
+      </c>
+      <c r="AD60" t="str">
+        <v>Iron Condor</v>
+      </c>
+      <c r="AE60">
+        <v>40</v>
+      </c>
+      <c r="AF60" t="str">
+        <v>Bull Call Spread</v>
+      </c>
+      <c r="AG60">
+        <v>25</v>
+      </c>
+      <c r="AH60">
+        <v>50000</v>
+      </c>
+      <c r="AI60" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AJ60" t="str">
+        <v>BUY 1030PE | SELL 1020PE</v>
+      </c>
+      <c r="AK60">
+        <v>1</v>
+      </c>
+      <c r="AL60">
+        <v>2.4</v>
+      </c>
+      <c r="AM60">
+        <v>2.16</v>
+      </c>
+      <c r="AN60">
+        <v>2.88</v>
+      </c>
+      <c r="AO60">
+        <v>180</v>
+      </c>
+      <c r="AP60">
+        <v>360</v>
+      </c>
+      <c r="AQ60">
+        <v>2</v>
+      </c>
+      <c r="AR60" t="str">
+        <v>scalp</v>
+      </c>
+      <c r="AS60" t="str">
+        <v>bias Bearish persisted 1/3 polls</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>2026-08-24 12:33:47</v>
+      </c>
+      <c r="B61">
+        <v>1035.2</v>
+      </c>
+      <c r="C61">
+        <v>1040</v>
+      </c>
+      <c r="D61">
+        <v>0.57</v>
+      </c>
+      <c r="E61">
+        <v>1000</v>
+      </c>
+      <c r="F61">
+        <v>1100</v>
+      </c>
+      <c r="G61">
+        <v>1080</v>
+      </c>
+      <c r="H61">
+        <v>1100</v>
+      </c>
+      <c r="I61">
+        <v>1080</v>
+      </c>
+      <c r="J61">
+        <v>1050</v>
+      </c>
+      <c r="K61">
+        <v>7</v>
+      </c>
+      <c r="L61">
+        <v>7</v>
+      </c>
+      <c r="M61">
+        <v>2160750</v>
+      </c>
+      <c r="N61">
+        <v>1787250</v>
+      </c>
+      <c r="O61" t="str">
+        <v>Put Unwinding 5x/1149750 | Call Covering 2x/1011000 | Put Covering 3x/448500 | Call Unwinding 4x/1338750</v>
+      </c>
+      <c r="P61">
+        <v>52.12</v>
+      </c>
+      <c r="Q61" t="str">
+        <v>Range</v>
+      </c>
+      <c r="R61">
+        <v>0.454</v>
+      </c>
+      <c r="S61">
+        <v>0.503</v>
+      </c>
+      <c r="T61">
+        <v>2.071</v>
+      </c>
+      <c r="U61">
+        <v>0.006</v>
+      </c>
+      <c r="V61">
+        <v>0.07</v>
+      </c>
+      <c r="W61" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X61">
+        <v>1038.8</v>
+      </c>
+      <c r="Y61">
+        <v>0.69</v>
+      </c>
+      <c r="Z61" t="str">
+        <v>Short Buildup</v>
+      </c>
+      <c r="AA61">
+        <v>83</v>
+      </c>
+      <c r="AB61" t="str">
+        <v>Iron Condor</v>
+      </c>
+      <c r="AC61">
+        <v>70</v>
+      </c>
+      <c r="AD61" t="str">
+        <v>Bull Call Spread</v>
+      </c>
+      <c r="AE61">
+        <v>50</v>
+      </c>
+      <c r="AF61" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AG61">
+        <v>50</v>
+      </c>
+      <c r="AH61">
+        <v>50000</v>
+      </c>
+      <c r="AI61" t="str">
+        <v>Iron Condor</v>
+      </c>
+      <c r="AJ61" t="str">
+        <v>SELL 1030PE | BUY 1020PE | SELL 1050CE | BUY 1060CE</v>
+      </c>
+      <c r="AK61">
+        <v>1</v>
+      </c>
+      <c r="AL61">
+        <v>-3.1</v>
+      </c>
+      <c r="AM61">
+        <v>-4.65</v>
+      </c>
+      <c r="AN61">
+        <v>0</v>
+      </c>
+      <c r="AO61">
+        <v>1163</v>
+      </c>
+      <c r="AP61">
+        <v>2325</v>
+      </c>
+      <c r="AQ61">
+        <v>2</v>
+      </c>
+      <c r="AR61" t="str">
+        <v>default</v>
+      </c>
+      <c r="AS61" t="str">
+        <v>bias Range persisted 1/3 polls</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AS59"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AS61"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
state: session end 2026-08-25T07:05Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -25491,7 +25491,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AS62"/>
+  <dimension ref="A1:AS63"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -32847,9 +32847,146 @@
         <v>NO TRADE</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>2026-08-25 12:33:30</v>
+      </c>
+      <c r="B63">
+        <v>1040.9</v>
+      </c>
+      <c r="C63">
+        <v>1040</v>
+      </c>
+      <c r="D63">
+        <v>0.93</v>
+      </c>
+      <c r="E63">
+        <v>1050</v>
+      </c>
+      <c r="F63">
+        <v>1000</v>
+      </c>
+      <c r="G63">
+        <v>1100</v>
+      </c>
+      <c r="H63">
+        <v>1100</v>
+      </c>
+      <c r="I63">
+        <v>1050</v>
+      </c>
+      <c r="J63">
+        <v>1060</v>
+      </c>
+      <c r="K63">
+        <v>6</v>
+      </c>
+      <c r="L63">
+        <v>17</v>
+      </c>
+      <c r="M63">
+        <v>884250</v>
+      </c>
+      <c r="N63">
+        <v>2916750</v>
+      </c>
+      <c r="O63" t="str">
+        <v>Call Writing 7x/1155750 | Put Buying 8x/1734750 | Call Buying 3x/732000 | Call Unwinding 2x/26250 | Put Writing 3x/152250</v>
+      </c>
+      <c r="P63">
+        <v>16.77</v>
+      </c>
+      <c r="Q63" t="str">
+        <v>Bearish</v>
+      </c>
+      <c r="R63">
+        <v>0.538</v>
+      </c>
+      <c r="S63">
+        <v>0.475</v>
+      </c>
+      <c r="T63">
+        <v>0.207</v>
+      </c>
+      <c r="U63">
+        <v>0.0044</v>
+      </c>
+      <c r="V63">
+        <v>0.818</v>
+      </c>
+      <c r="W63" t="str">
+        <v>Down</v>
+      </c>
+      <c r="X63">
+        <v>1039.03</v>
+      </c>
+      <c r="Y63">
+        <v>0.74</v>
+      </c>
+      <c r="Z63" t="str">
+        <v>Short Buildup</v>
+      </c>
+      <c r="AA63">
+        <v>83</v>
+      </c>
+      <c r="AB63" t="str">
+        <v>Buy Put</v>
+      </c>
+      <c r="AC63">
+        <v>100</v>
+      </c>
+      <c r="AD63" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AE63">
+        <v>100</v>
+      </c>
+      <c r="AF63" t="str">
+        <v>Iron Condor</v>
+      </c>
+      <c r="AG63">
+        <v>30</v>
+      </c>
+      <c r="AH63">
+        <v>50000</v>
+      </c>
+      <c r="AI63" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AJ63" t="str">
+        <v>BUY 1040PE | SELL 1030PE</v>
+      </c>
+      <c r="AK63">
+        <v>1</v>
+      </c>
+      <c r="AL63">
+        <v>4</v>
+      </c>
+      <c r="AM63">
+        <v>2</v>
+      </c>
+      <c r="AN63" t="str">
+        <v>SIGNAL</v>
+      </c>
+      <c r="AO63">
+        <v>1500</v>
+      </c>
+      <c r="AP63" t="str">
+        <v/>
+      </c>
+      <c r="AQ63" t="str">
+        <v/>
+      </c>
+      <c r="AR63" t="str">
+        <v>ride</v>
+      </c>
+      <c r="AS63" t="str">
+        <v>bias Bearish persisted 1/3 polls</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AS62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AS63"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>